<commit_message>
Nitar 01 ke Wilayah Segamat (3/2/1/3), buang Kalabakan
- data.js: Nitar 01 no. 11 di Segamat, Kalabakan dikeluarkan; jumlah kekal 97/62/31/126
- Tracking xlsx: baris Kalabakan dibuang, Nitar 01 dimasukkan dalam Segamat,
  merged cell wilayah & nombor BIL dikemas kini
- RANCANGAN xlsx: Nitar 01 dialih dari kumpulan Johor Bahru ke Segamat
- PLANNING.md dikemas kini

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/RANCANGAN_FELDA_KIT_GAJAH_2026.xlsx
+++ b/RANCANGAN_FELDA_KIT_GAJAH_2026.xlsx
@@ -829,7 +829,7 @@
       </c>
     </row>
     <row r="13" spans="2:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="3"/>
+      <c r="B13" s="2"/>
       <c r="C13" s="9">
         <v>10</v>
       </c>
@@ -838,7 +838,9 @@
       </c>
     </row>
     <row r="14" spans="2:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="2"/>
+      <c r="B14" s="1" t="s">
+        <v>14</v>
+      </c>
       <c r="C14" s="9">
         <v>11</v>
       </c>
@@ -847,9 +849,7 @@
       </c>
     </row>
     <row r="15" spans="2:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="1" t="s">
-        <v>14</v>
-      </c>
+      <c r="B15" s="3"/>
       <c r="C15" s="9">
         <v>12</v>
       </c>
@@ -1149,9 +1149,9 @@
     <mergeCell ref="B23:B29"/>
     <mergeCell ref="B30:B33"/>
     <mergeCell ref="B34:B36"/>
-    <mergeCell ref="B15:B20"/>
+    <mergeCell ref="B14:B20"/>
     <mergeCell ref="B21:B22"/>
-    <mergeCell ref="B4:B14"/>
+    <mergeCell ref="B4:B13"/>
     <mergeCell ref="B2:B3"/>
     <mergeCell ref="C2:C3"/>
     <mergeCell ref="D2:D3"/>

</xml_diff>